<commit_message>
Add contract days prediction pipeline
</commit_message>
<xml_diff>
--- a/data/input/prediction_input.xlsx
+++ b/data/input/prediction_input.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -60,13 +62,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -450,6 +453,10 @@
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,6 +535,26 @@
           <t>asking_price</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>station_name</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>station_line</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>station_latitude</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>station_longitude</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -591,6 +618,22 @@
       <c r="O2" s="3" t="n">
         <v>45000000</v>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>北千住</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>常磐線</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>35.74929865138866</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>139.8050594329834</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -654,6 +697,22 @@
       <c r="O3" s="3" t="n">
         <v>60000000</v>
       </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>三軒茶屋</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>田園都市線</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>35.64366111008705</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>139.6712923049927</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -716,6 +775,22 @@
       </c>
       <c r="O4" s="3" t="n">
         <v>120000000</v>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>六本木</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>2号線日比谷線</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>35.66329357678096</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>139.7321462631226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>